<commit_message>
pelipaikat updated 18.10 added
</commit_message>
<xml_diff>
--- a/pelipaikat.xlsx
+++ b/pelipaikat.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\own_prog\github\kaudet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28B83B2D-C855-4DC9-827E-6CCFEEDC323D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5DD2741-4A69-416A-9860-21289772963C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{4555F0EC-1DB6-484D-B801-2FC196B7544F}"/>
   </bookViews>
@@ -474,7 +474,7 @@
     <t>Vapaa-aikakeskus</t>
   </si>
   <si>
-    <t>3.10.2026</t>
+    <t>18.10.2026</t>
   </si>
 </sst>
 </file>
@@ -1114,18 +1114,20 @@
       <c r="K4" s="8"/>
       <c r="L4" s="8"/>
       <c r="M4" s="8"/>
-      <c r="N4" s="8"/>
+      <c r="N4" s="8">
+        <v>1</v>
+      </c>
       <c r="O4" s="8">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P4" s="8">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Q4" s="8">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="R4" s="8"/>
     </row>
@@ -3473,18 +3475,20 @@
       <c r="K57" s="14"/>
       <c r="L57" s="14"/>
       <c r="M57" s="14"/>
-      <c r="N57" s="14"/>
+      <c r="N57" s="14">
+        <v>1</v>
+      </c>
       <c r="O57" s="14">
         <f t="shared" si="2"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P57" s="14">
         <f t="shared" si="4"/>
-        <v>130</v>
+        <v>195</v>
       </c>
       <c r="Q57" s="14">
         <f t="shared" si="1"/>
-        <v>260</v>
+        <v>390</v>
       </c>
       <c r="R57" s="14"/>
     </row>
@@ -4082,15 +4086,15 @@
       <c r="N71" s="6"/>
       <c r="O71" s="6">
         <f>SUM(O2:O70)</f>
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="P71" s="6">
         <f>SUM(P2:P70)</f>
-        <v>13282</v>
+        <v>13351</v>
       </c>
       <c r="Q71" s="6">
         <f>SUM(Q2:Q70)</f>
-        <v>26564</v>
+        <v>26702</v>
       </c>
       <c r="R71" s="6"/>
     </row>
@@ -4148,7 +4152,7 @@
       <c r="P72" s="12"/>
       <c r="Q72" s="7">
         <f>SUM(Q2:Q70)</f>
-        <v>26564</v>
+        <v>26702</v>
       </c>
       <c r="R72" s="13">
         <f>SUM(R2:R70)</f>
@@ -4446,7 +4450,7 @@
       </c>
       <c r="R83" s="8">
         <f>SUM(Q83:Q86)</f>
-        <v>148</v>
+        <v>156</v>
       </c>
     </row>
     <row r="84" spans="1:18" x14ac:dyDescent="0.3">
@@ -4565,13 +4569,13 @@
       </c>
       <c r="N85" s="8">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="O85" s="8"/>
       <c r="P85" s="8"/>
       <c r="Q85" s="8">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="R85" s="8"/>
     </row>
@@ -8092,7 +8096,7 @@
       </c>
       <c r="R137" s="14">
         <f>SUM(Q137:Q139)</f>
-        <v>1004</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="138" spans="1:31" s="17" customFormat="1" x14ac:dyDescent="0.3">
@@ -8148,13 +8152,13 @@
       </c>
       <c r="N138" s="14">
         <f t="shared" si="37"/>
-        <v>0</v>
+        <v>130</v>
       </c>
       <c r="O138" s="14"/>
       <c r="P138" s="14"/>
       <c r="Q138" s="14">
         <f t="shared" si="12"/>
-        <v>260</v>
+        <v>390</v>
       </c>
       <c r="R138" s="14"/>
     </row>
@@ -9146,23 +9150,23 @@
       </c>
       <c r="N155" s="8">
         <f t="shared" si="51"/>
-        <v>584</v>
+        <v>722</v>
       </c>
       <c r="O155" s="8">
         <f>SUM(D155:N155)</f>
-        <v>26564</v>
+        <v>26702</v>
       </c>
       <c r="P155" s="15">
         <f>O155/O72</f>
-        <v>158.11904761904762</v>
+        <v>158.9404761904762</v>
       </c>
       <c r="Q155" s="8">
         <f>SUM(Q83:Q151)</f>
-        <v>26564</v>
+        <v>26702</v>
       </c>
       <c r="R155" s="8">
         <f>SUM(R83:R151)</f>
-        <v>26564</v>
+        <v>26702</v>
       </c>
     </row>
     <row r="156" spans="1:31" x14ac:dyDescent="0.3">
@@ -9215,7 +9219,7 @@
       </c>
       <c r="O156" s="16">
         <f t="shared" si="52"/>
-        <v>158.11904761904762</v>
+        <v>158.9404761904762</v>
       </c>
       <c r="P156" s="6" t="s">
         <v>97</v>
@@ -9247,11 +9251,11 @@
       </c>
       <c r="C160" s="8">
         <f>SUM(O2:O5)</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D160" s="8">
         <f>R83</f>
-        <v>148</v>
+        <v>156</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.3">
@@ -9672,11 +9676,11 @@
       </c>
       <c r="C185" s="14">
         <f>SUM(O56:O58)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D185" s="14">
         <f>R137</f>
-        <v>1004</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="186" spans="1:4" x14ac:dyDescent="0.3">
@@ -9789,11 +9793,11 @@
       </c>
       <c r="C192" s="20">
         <f>SUM(C160:C191)</f>
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D192" s="20">
         <f>SUM(D160:D191)</f>
-        <v>26188</v>
+        <v>26326</v>
       </c>
     </row>
   </sheetData>

</xml_diff>